<commit_message>
feat(story-4.1): Tạo Đơn + dựng giỏ hàng + snapshot Order.sourceId (Order/OrderVersion/OrderLineItem)
</commit_message>
<xml_diff>
--- a/_bmad-output/planning-artifacts/bao-gia-phat-trien-app-phuong-nam-solar-phase1.xlsx
+++ b/_bmad-output/planning-artifacts/bao-gia-phat-trien-app-phuong-nam-solar-phase1.xlsx
@@ -153,7 +153,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -175,11 +175,55 @@
         <color rgb="00C9D6D2"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9D6D2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9D6D2"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9D6D2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9D6D2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9D6D2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9D6D2"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9D6D2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9D6D2"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -264,6 +308,8 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -629,7 +675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D97"/>
+  <dimension ref="A1:D119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -679,7 +725,7 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Số BG: BG-DEV-2026-001</t>
+          <t>Số BG: BG-DEV-2026-001-A</t>
         </is>
       </c>
     </row>
@@ -696,7 +742,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Ngày: …/…/2026</t>
+          <t>Ngày: …/…/2026 (cập nhật 13/07)</t>
         </is>
       </c>
     </row>
@@ -745,8 +791,8 @@
           <t>0. Khởi tạo &amp; Nền tảng</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="9" t="n"/>
+      <c r="B12" s="34" t="n"/>
+      <c r="C12" s="35" t="n"/>
       <c r="D12" s="10">
         <f>SUM(D13:D17)</f>
         <v/>
@@ -848,8 +894,8 @@
           <t>1. Xác thực &amp; Tài khoản</t>
         </is>
       </c>
-      <c r="B18" s="9" t="n"/>
-      <c r="C18" s="9" t="n"/>
+      <c r="B18" s="34" t="n"/>
+      <c r="C18" s="35" t="n"/>
       <c r="D18" s="10">
         <f>SUM(D19:D21)</f>
         <v/>
@@ -915,8 +961,8 @@
           <t>2. Khách hàng</t>
         </is>
       </c>
-      <c r="B22" s="9" t="n"/>
-      <c r="C22" s="9" t="n"/>
+      <c r="B22" s="34" t="n"/>
+      <c r="C22" s="35" t="n"/>
       <c r="D22" s="10">
         <f>SUM(D23:D24)</f>
         <v/>
@@ -964,8 +1010,8 @@
           <t>3. Danh mục vật tư &amp; Giá</t>
         </is>
       </c>
-      <c r="B25" s="9" t="n"/>
-      <c r="C25" s="9" t="n"/>
+      <c r="B25" s="34" t="n"/>
+      <c r="C25" s="35" t="n"/>
       <c r="D25" s="10">
         <f>SUM(D26:D27)</f>
         <v/>
@@ -1013,8 +1059,8 @@
           <t>4. Báo giá &amp; Đơn hàng (lõi)</t>
         </is>
       </c>
-      <c r="B28" s="9" t="n"/>
-      <c r="C28" s="9" t="n"/>
+      <c r="B28" s="34" t="n"/>
+      <c r="C28" s="35" t="n"/>
       <c r="D28" s="10">
         <f>SUM(D29:D35)</f>
         <v/>
@@ -1152,8 +1198,8 @@
           <t>5. Vòng đời &amp; Trạng thái đơn</t>
         </is>
       </c>
-      <c r="B36" s="9" t="n"/>
-      <c r="C36" s="9" t="n"/>
+      <c r="B36" s="34" t="n"/>
+      <c r="C36" s="35" t="n"/>
       <c r="D36" s="10">
         <f>SUM(D37:D41)</f>
         <v/>
@@ -1255,8 +1301,8 @@
           <t>6. Đính kèm ảnh</t>
         </is>
       </c>
-      <c r="B42" s="9" t="n"/>
-      <c r="C42" s="9" t="n"/>
+      <c r="B42" s="34" t="n"/>
+      <c r="C42" s="35" t="n"/>
       <c r="D42" s="10">
         <f>SUM(D43:D43)</f>
         <v/>
@@ -1286,8 +1332,8 @@
           <t>7. Thanh toán</t>
         </is>
       </c>
-      <c r="B44" s="9" t="n"/>
-      <c r="C44" s="9" t="n"/>
+      <c r="B44" s="34" t="n"/>
+      <c r="C44" s="35" t="n"/>
       <c r="D44" s="10">
         <f>SUM(D45:D46)</f>
         <v/>
@@ -1335,8 +1381,8 @@
           <t>8. Hợp đồng &amp; Hoá đơn</t>
         </is>
       </c>
-      <c r="B47" s="9" t="n"/>
-      <c r="C47" s="9" t="n"/>
+      <c r="B47" s="34" t="n"/>
+      <c r="C47" s="35" t="n"/>
       <c r="D47" s="10">
         <f>SUM(D48:D49)</f>
         <v/>
@@ -1384,8 +1430,8 @@
           <t>9. Tồn kho</t>
         </is>
       </c>
-      <c r="B50" s="9" t="n"/>
-      <c r="C50" s="9" t="n"/>
+      <c r="B50" s="34" t="n"/>
+      <c r="C50" s="35" t="n"/>
       <c r="D50" s="10">
         <f>SUM(D51:D52)</f>
         <v/>
@@ -1433,8 +1479,8 @@
           <t>10. Phân quyền &amp; Duyệt</t>
         </is>
       </c>
-      <c r="B53" s="9" t="n"/>
-      <c r="C53" s="9" t="n"/>
+      <c r="B53" s="34" t="n"/>
+      <c r="C53" s="35" t="n"/>
       <c r="D53" s="10">
         <f>SUM(D54:D56)</f>
         <v/>
@@ -1500,8 +1546,8 @@
           <t>11. Dashboard &amp; Báo cáo</t>
         </is>
       </c>
-      <c r="B57" s="9" t="n"/>
-      <c r="C57" s="9" t="n"/>
+      <c r="B57" s="34" t="n"/>
+      <c r="C57" s="35" t="n"/>
       <c r="D57" s="10">
         <f>SUM(D58:D58)</f>
         <v/>
@@ -1531,8 +1577,8 @@
           <t>12. Audit log</t>
         </is>
       </c>
-      <c r="B59" s="9" t="n"/>
-      <c r="C59" s="9" t="n"/>
+      <c r="B59" s="34" t="n"/>
+      <c r="C59" s="35" t="n"/>
       <c r="D59" s="10">
         <f>SUM(D60:D60)</f>
         <v/>
@@ -1562,8 +1608,8 @@
           <t>13. QA, Tài liệu &amp; Bàn giao</t>
         </is>
       </c>
-      <c r="B61" s="9" t="n"/>
-      <c r="C61" s="9" t="n"/>
+      <c r="B61" s="34" t="n"/>
+      <c r="C61" s="35" t="n"/>
       <c r="D61" s="10">
         <f>SUM(D62:D64)</f>
         <v/>
@@ -1629,8 +1675,8 @@
           <t>14. Thiết kế, triển khai &amp; mục bổ sung</t>
         </is>
       </c>
-      <c r="B65" s="9" t="n"/>
-      <c r="C65" s="9" t="n"/>
+      <c r="B65" s="34" t="n"/>
+      <c r="C65" s="35" t="n"/>
       <c r="D65" s="10">
         <f>SUM(D66:D69)</f>
         <v/>
@@ -1708,355 +1754,702 @@
         <v>3000000</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="14" t="inlineStr">
-        <is>
-          <t>Cộng chi phí phát triển</t>
-        </is>
-      </c>
-      <c r="B71" s="15" t="n"/>
-      <c r="C71" s="15" t="n"/>
-      <c r="D71" s="13">
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="7" t="inlineStr">
+        <is>
+          <t>PHỤ LỤC A — PHÁT SINH THEO YÊU CẦU KHÁCH HÀNG (10/07/2026)</t>
+        </is>
+      </c>
+      <c r="B71" s="34" t="n"/>
+      <c r="C71" s="34" t="n"/>
+      <c r="D71" s="35" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="inlineStr">
+        <is>
+          <t>A1. Nguồn khách &amp; Gói vật tư</t>
+        </is>
+      </c>
+      <c r="B72" s="34" t="n"/>
+      <c r="C72" s="35" t="n"/>
+      <c r="D72" s="10">
+        <f>SUM(D73:D74)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="26" customHeight="1">
+      <c r="A73" s="11" t="n">
+        <v>44</v>
+      </c>
+      <c r="B73" s="12" t="inlineStr">
+        <is>
+          <t>Nguồn khách hàng</t>
+        </is>
+      </c>
+      <c r="C73" s="12" t="inlineStr">
+        <is>
+          <t>Danh mục nguồn (Facebook/Zalo/Fanpage/Đại lý/Khác) + màn cấu hình; gắn nguồn lên khách; đơn snapshot nguồn lúc tạo</t>
+        </is>
+      </c>
+      <c r="D73" s="13" t="n">
+        <v>3600000</v>
+      </c>
+    </row>
+    <row r="74" ht="26" customHeight="1">
+      <c r="A74" s="11" t="n">
+        <v>45</v>
+      </c>
+      <c r="B74" s="12" t="inlineStr">
+        <is>
+          <t>Gói vật tư (checklist)</t>
+        </is>
+      </c>
+      <c r="C74" s="12" t="inlineStr">
+        <is>
+          <t>Nhóm sản phẩm dạng checklist; tick item → sinh dòng báo giá trỏ sản phẩm thật</t>
+        </is>
+      </c>
+      <c r="D74" s="13" t="n">
+        <v>3600000</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
+          <t>A2. Bảo hành</t>
+        </is>
+      </c>
+      <c r="B75" s="34" t="n"/>
+      <c r="C75" s="35" t="n"/>
+      <c r="D75" s="10">
+        <f>SUM(D76:D77)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76" ht="26" customHeight="1">
+      <c r="A76" s="11" t="n">
+        <v>46</v>
+      </c>
+      <c r="B76" s="12" t="inlineStr">
+        <is>
+          <t>Bảo hành theo dòng vật tư</t>
+        </is>
+      </c>
+      <c r="C76" s="12" t="inlineStr">
+        <is>
+          <t>Bảo hành mặc định trên sản phẩm, sửa được trên dòng, đóng băng lúc chốt; thêm cột Bảo hành vào PDF báo giá</t>
+        </is>
+      </c>
+      <c r="D76" s="13" t="n">
+        <v>3000000</v>
+      </c>
+    </row>
+    <row r="77" ht="26" customHeight="1">
+      <c r="A77" s="11" t="n">
+        <v>47</v>
+      </c>
+      <c r="B77" s="12" t="inlineStr">
+        <is>
+          <t>Tra cứu bảo hành theo SĐT</t>
+        </is>
+      </c>
+      <c r="C77" s="12" t="inlineStr">
+        <is>
+          <t>Tra SĐT → đơn → từng vật tư kèm hạn còn lại (web + mobile)</t>
+        </is>
+      </c>
+      <c r="D77" s="13" t="n">
+        <v>3600000</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="8" t="inlineStr">
+        <is>
+          <t>A3. Tồn kho &amp; Giá vốn</t>
+        </is>
+      </c>
+      <c r="B78" s="34" t="n"/>
+      <c r="C78" s="35" t="n"/>
+      <c r="D78" s="10">
+        <f>SUM(D79:D81)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79" ht="26" customHeight="1">
+      <c r="A79" s="11" t="n">
+        <v>48</v>
+      </c>
+      <c r="B79" s="12" t="inlineStr">
+        <is>
+          <t>Tồn kho hai con số (tồn thật / đã hứa / khả dụng)</t>
+        </is>
+      </c>
+      <c r="C79" s="12" t="inlineStr">
+        <is>
+          <t>Sổ giữ chỗ khi chốt đơn, cảnh báo sớm ngay lúc thêm dòng, tổng hợp danh sách cần mua</t>
+        </is>
+      </c>
+      <c r="D79" s="13" t="n">
+        <v>7200000</v>
+      </c>
+    </row>
+    <row r="80" ht="26" customHeight="1">
+      <c r="A80" s="11" t="n">
+        <v>49</v>
+      </c>
+      <c r="B80" s="12" t="inlineStr">
+        <is>
+          <t>Phiếu nhập trả khi huỷ đơn đã xuất</t>
+        </is>
+      </c>
+      <c r="C80" s="12" t="inlineStr">
+        <is>
+          <t>Huỷ sau khi xuất kho → phiếu nhập trả để hoàn tồn, không tự cộng ngầm</t>
+        </is>
+      </c>
+      <c r="D80" s="13" t="n">
+        <v>2400000</v>
+      </c>
+    </row>
+    <row r="81" ht="26" customHeight="1">
+      <c r="A81" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="B81" s="12" t="inlineStr">
+        <is>
+          <t>Giá vốn nhập &amp; bình quân gia quyền</t>
+        </is>
+      </c>
+      <c r="C81" s="12" t="inlineStr">
+        <is>
+          <t>Bắt buộc giá vốn trên phiếu nhập → tự tính bình quân gia quyền → đóng băng giá vốn lúc xuất kho</t>
+        </is>
+      </c>
+      <c r="D81" s="13" t="n">
+        <v>3600000</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="inlineStr">
+        <is>
+          <t>A4. Báo cáo</t>
+        </is>
+      </c>
+      <c r="B82" s="34" t="n"/>
+      <c r="C82" s="35" t="n"/>
+      <c r="D82" s="10">
+        <f>SUM(D83:D84)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83" ht="26" customHeight="1">
+      <c r="A83" s="11" t="n">
+        <v>51</v>
+      </c>
+      <c r="B83" s="12" t="inlineStr">
+        <is>
+          <t>Báo cáo lợi nhuận gộp</t>
+        </is>
+      </c>
+      <c r="C83" s="12" t="inlineStr">
+        <is>
+          <t>Một bảng, bốn cách nhóm: theo đơn / tháng / sale / nguồn khách; kèm dòng KPI</t>
+        </is>
+      </c>
+      <c r="D83" s="13" t="n">
+        <v>6000000</v>
+      </c>
+    </row>
+    <row r="84" ht="26" customHeight="1">
+      <c r="A84" s="11" t="n">
+        <v>52</v>
+      </c>
+      <c r="B84" s="12" t="inlineStr">
+        <is>
+          <t>Báo cáo công nợ</t>
+        </is>
+      </c>
+      <c r="C84" s="12" t="inlineStr">
+        <is>
+          <t>Đã thu / còn nợ / quá hạn theo đơn và theo khách; kèm dòng KPI</t>
+        </is>
+      </c>
+      <c r="D84" s="13" t="n">
+        <v>4800000</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="inlineStr">
+        <is>
+          <t>A5. Quyền &amp; Trạng thái đơn</t>
+        </is>
+      </c>
+      <c r="B85" s="34" t="n"/>
+      <c r="C85" s="35" t="n"/>
+      <c r="D85" s="10">
+        <f>SUM(D86:D87)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86" ht="26" customHeight="1">
+      <c r="A86" s="11" t="n">
+        <v>53</v>
+      </c>
+      <c r="B86" s="12" t="inlineStr">
+        <is>
+          <t>Ba quyền mới + luật chống leo thang quyền</t>
+        </is>
+      </c>
+      <c r="C86" s="12" t="inlineStr">
+        <is>
+          <t>Cấu hình hệ thống, cờ tính năng, xem giá vốn; chặn tự cấp quyền mình không có</t>
+        </is>
+      </c>
+      <c r="D86" s="13" t="n">
+        <v>3000000</v>
+      </c>
+    </row>
+    <row r="87" ht="26" customHeight="1">
+      <c r="A87" s="11" t="n">
+        <v>54</v>
+      </c>
+      <c r="B87" s="12" t="inlineStr">
+        <is>
+          <t>Trạng thái "Đã giao" + bỏ bước "Lên lịch thi công"</t>
+        </is>
+      </c>
+      <c r="C87" s="12" t="inlineStr">
+        <is>
+          <t>Bổ sung trạng thái Đã giao gate theo cờ Thiết bị; cập nhật máy trạng thái, web và mobile</t>
+        </is>
+      </c>
+      <c r="D87" s="13" t="n">
+        <v>1800000</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="8" t="inlineStr">
+        <is>
+          <t>A6. Thiết kế bổ sung</t>
+        </is>
+      </c>
+      <c r="B88" s="34" t="n"/>
+      <c r="C88" s="35" t="n"/>
+      <c r="D88" s="10">
+        <f>SUM(D89:D89)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89" ht="26" customHeight="1">
+      <c r="A89" s="11" t="n">
+        <v>55</v>
+      </c>
+      <c r="B89" s="12" t="inlineStr">
+        <is>
+          <t>Thiết kế UI/UX các màn phát sinh</t>
+        </is>
+      </c>
+      <c r="C89" s="12" t="inlineStr">
+        <is>
+          <t>5 màn mới + cập nhật 8 màn hiện có (25 → 30 màn)</t>
+        </is>
+      </c>
+      <c r="D89" s="13" t="n">
+        <v>3000000</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="14" t="inlineStr">
+        <is>
+          <t>Cộng hạng mục gốc (mục 1–43)</t>
+        </is>
+      </c>
+      <c r="B91" s="34" t="n"/>
+      <c r="C91" s="35" t="n"/>
+      <c r="D91" s="13">
         <f>D12+D18+D22+D25+D28+D36+D42+D44+D47+D50+D53+D57+D59+D61+D65</f>
         <v/>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="14" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="14" t="inlineStr">
+        <is>
+          <t>Cộng phụ lục phát sinh (mục 44–55)</t>
+        </is>
+      </c>
+      <c r="B92" s="34" t="n"/>
+      <c r="C92" s="35" t="n"/>
+      <c r="D92" s="13">
+        <f>D72+D75+D78+D82+D85+D88</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="17" t="inlineStr">
+        <is>
+          <t>TỔNG CHI PHÍ PHÁT TRIỂN</t>
+        </is>
+      </c>
+      <c r="B93" s="34" t="n"/>
+      <c r="C93" s="35" t="n"/>
+      <c r="D93" s="19">
+        <f>D91+D92</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="14" t="inlineStr">
         <is>
           <t>Dự phòng rủi ro (12%)</t>
         </is>
       </c>
-      <c r="B72" s="15" t="n"/>
-      <c r="C72" s="15" t="n"/>
-      <c r="D72" s="16">
-        <f>D71*0.12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="17" t="inlineStr">
+      <c r="B94" s="34" t="n"/>
+      <c r="C94" s="35" t="n"/>
+      <c r="D94" s="13">
+        <f>D93*0.12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="17" t="inlineStr">
         <is>
           <t>TỔNG CỘNG (trước VAT)</t>
         </is>
       </c>
-      <c r="B73" s="18" t="n"/>
-      <c r="C73" s="18" t="n"/>
-      <c r="D73" s="19">
-        <f>D71+D72</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="14" t="inlineStr">
+      <c r="B95" s="34" t="n"/>
+      <c r="C95" s="35" t="n"/>
+      <c r="D95" s="19">
+        <f>D93+D94</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="14" t="inlineStr">
         <is>
           <t>Thuế VAT (8%)</t>
         </is>
       </c>
-      <c r="B74" s="15" t="n"/>
-      <c r="C74" s="15" t="n"/>
-      <c r="D74" s="16">
-        <f>D73*0.08</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75" ht="24" customHeight="1">
-      <c r="A75" s="20" t="inlineStr">
+      <c r="B96" s="34" t="n"/>
+      <c r="C96" s="35" t="n"/>
+      <c r="D96" s="13">
+        <f>D95*0.08</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97" ht="24" customHeight="1">
+      <c r="A97" s="20" t="inlineStr">
         <is>
           <t>TỔNG CỘNG (sau VAT)</t>
         </is>
       </c>
-      <c r="B75" s="21" t="n"/>
-      <c r="C75" s="21" t="n"/>
-      <c r="D75" s="22">
-        <f>D73+D74</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="23" t="inlineStr">
+      <c r="B97" s="34" t="n"/>
+      <c r="C97" s="35" t="n"/>
+      <c r="D97" s="22">
+        <f>D95+D96</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="23" t="inlineStr">
         <is>
           <t>GHI CHÚ &amp; PHẠM VI</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="26" customHeight="1">
-      <c r="A78" s="24" t="inlineStr">
-        <is>
-          <t>• Báo giá trọn gói theo từng hạng mục. Đã bao gồm: phân tích, thiết kế UI (mockup 25 màn), lập trình Web + Mobile + Backend, kiểm thử, tài liệu, triển khai, phân phối app và dự phòng rủi ro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="26" customHeight="1">
-      <c r="A79" s="24" t="inlineStr">
-        <is>
-          <t>• Chưa bao gồm (báo giá riêng khi phát sinh): cổng đại lý tự đặt hàng, tích hợp hoá đơn điện tử nhà cung cấp (VNPT/Viettel…), CRM đầy đủ, offline mode, quản lý nhiều kho.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="26" customHeight="1">
-      <c r="A80" s="24" t="inlineStr">
+    <row r="100" ht="26" customHeight="1">
+      <c r="A100" s="24" t="inlineStr">
+        <is>
+          <t>• Báo giá trọn gói theo từng hạng mục. Đã bao gồm: phân tích, thiết kế UI (mockup 30 màn), lập trình Web + Mobile + Backend, kiểm thử, tài liệu, triển khai, phân phối app và dự phòng rủi ro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="26" customHeight="1">
+      <c r="A101" s="24" t="inlineStr">
+        <is>
+          <t>• Chưa bao gồm (báo giá riêng khi phát sinh): cổng đại lý tự đặt hàng, tích hợp hoá đơn điện tử nhà cung cấp (VNPT/Viettel…), CRM đầy đủ, offline mode, quản lý nhiều kho, phiếu yêu cầu bảo hành &amp; nhắc hết hạn, BOM/định mức vật tư, truy vết serial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="26" customHeight="1">
+      <c r="A102" s="24" t="inlineStr">
         <is>
           <t>• Chi phí HÀNG THÁNG/định kỳ sau bàn giao (bảo trì, VPS, SMS, tên miền, tài khoản Apple/Google): xem bảng bên dưới; KHÔNG tính trong tổng báo giá trên.</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="26" customHeight="1">
-      <c r="A81" s="24" t="inlineStr">
+    <row r="103" ht="26" customHeight="1">
+      <c r="A103" s="24" t="inlineStr">
         <is>
           <t>• Bảo trì, hỗ trợ &amp; nâng cấp sau bàn giao: theo phí hàng tháng (bảng bên dưới) hoặc hợp đồng riêng.</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="26" customHeight="1">
-      <c r="A82" s="24" t="inlineStr">
+    <row r="104" ht="26" customHeight="1">
+      <c r="A104" s="24" t="inlineStr">
+        <is>
+          <t>• Phụ lục A là các hạng mục khách hàng bổ sung ngày 10/07/2026, báo giá riêng từng dòng để tiện đối chiếu và điều chỉnh phạm vi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="24" t="inlineStr">
         <is>
           <t>• Thanh toán theo tiến độ hợp đồng — đề xuất chia đợt theo nhóm hạng mục.</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="23" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="23" t="inlineStr">
         <is>
           <t>CHI PHÍ HÀNG THÁNG / ĐỊNH KỲ (sau bàn giao — KHÔNG gồm trong tổng báo giá trên)</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="25" t="inlineStr">
+    <row r="107">
+      <c r="A107" s="25" t="inlineStr">
         <is>
           <t>Hạng mục</t>
         </is>
       </c>
-      <c r="B85" s="26" t="n"/>
-      <c r="C85" s="25" t="inlineStr">
+      <c r="B107" s="35" t="n"/>
+      <c r="C107" s="25" t="inlineStr">
         <is>
           <t>Chi phí / chu kỳ</t>
         </is>
       </c>
-      <c r="D85" s="25" t="inlineStr">
+      <c r="D107" s="25" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="18" customHeight="1">
-      <c r="A86" s="27" t="inlineStr">
+    <row r="108" ht="18" customHeight="1">
+      <c r="A108" s="27" t="inlineStr">
         <is>
           <t>Phí bảo trì &amp; hỗ trợ phần mềm</t>
         </is>
       </c>
-      <c r="B86" s="21" t="n"/>
-      <c r="C86" s="28" t="inlineStr">
+      <c r="B108" s="35" t="n"/>
+      <c r="C108" s="28" t="inlineStr">
         <is>
           <t>5.000.000 đ / tháng</t>
         </is>
       </c>
-      <c r="D86" s="29" t="inlineStr">
+      <c r="D108" s="29" t="inlineStr">
         <is>
           <t>Sửa lỗi, cập nhật nhỏ, hỗ trợ vận hành — tính từ sau bàn giao</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="18" customHeight="1">
-      <c r="A87" s="30" t="inlineStr">
+    <row r="109" ht="18" customHeight="1">
+      <c r="A109" s="30" t="inlineStr">
         <is>
           <t>Thuê máy chủ VPS</t>
         </is>
       </c>
-      <c r="B87" s="15" t="n"/>
-      <c r="C87" s="31" t="inlineStr">
+      <c r="B109" s="35" t="n"/>
+      <c r="C109" s="31" t="inlineStr">
         <is>
           <t>~500.000 đ / tháng</t>
         </is>
       </c>
-      <c r="D87" s="30" t="inlineStr">
+      <c r="D109" s="30" t="inlineStr">
         <is>
           <t>Tuỳ cấu hình máy chủ</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="18" customHeight="1">
-      <c r="A88" s="30" t="inlineStr">
+    <row r="110" ht="18" customHeight="1">
+      <c r="A110" s="30" t="inlineStr">
         <is>
           <t>SMS OTP (quên mật khẩu)</t>
         </is>
       </c>
-      <c r="B88" s="15" t="n"/>
-      <c r="C88" s="31" t="inlineStr">
+      <c r="B110" s="35" t="n"/>
+      <c r="C110" s="31" t="inlineStr">
         <is>
           <t>~500 đ / tin</t>
         </is>
       </c>
-      <c r="D88" s="30" t="inlineStr">
+      <c r="D110" s="30" t="inlineStr">
         <is>
           <t>Theo lượng tin gửi thực tế</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="18" customHeight="1">
-      <c r="A89" s="30" t="inlineStr">
+    <row r="111" ht="18" customHeight="1">
+      <c r="A111" s="30" t="inlineStr">
         <is>
           <t>Tên miền</t>
         </is>
       </c>
-      <c r="B89" s="15" t="n"/>
-      <c r="C89" s="31" t="inlineStr">
+      <c r="B111" s="35" t="n"/>
+      <c r="C111" s="31" t="inlineStr">
         <is>
           <t>~300.000 đ / năm</t>
         </is>
       </c>
-      <c r="D89" s="30" t="inlineStr">
+      <c r="D111" s="30" t="inlineStr">
         <is>
           <t>.vn/.com — gia hạn hằng năm</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="18" customHeight="1">
-      <c r="A90" s="30" t="inlineStr">
+    <row r="112" ht="18" customHeight="1">
+      <c r="A112" s="30" t="inlineStr">
         <is>
           <t>Chứng chỉ SSL</t>
         </is>
       </c>
-      <c r="B90" s="15" t="n"/>
-      <c r="C90" s="31" t="inlineStr">
+      <c r="B112" s="35" t="n"/>
+      <c r="C112" s="31" t="inlineStr">
         <is>
           <t>Miễn phí</t>
         </is>
       </c>
-      <c r="D90" s="30" t="inlineStr">
+      <c r="D112" s="30" t="inlineStr">
         <is>
           <t>Let's Encrypt</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="18" customHeight="1">
-      <c r="A91" s="30" t="inlineStr">
+    <row r="113" ht="18" customHeight="1">
+      <c r="A113" s="30" t="inlineStr">
         <is>
           <t>Tài khoản Apple Developer</t>
         </is>
       </c>
-      <c r="B91" s="15" t="n"/>
-      <c r="C91" s="31" t="inlineStr">
+      <c r="B113" s="35" t="n"/>
+      <c r="C113" s="31" t="inlineStr">
         <is>
           <t>~2.500.000 đ / năm</t>
         </is>
       </c>
-      <c r="D91" s="30" t="inlineStr">
+      <c r="D113" s="30" t="inlineStr">
         <is>
           <t>Nếu phát hành App Store</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="18" customHeight="1">
-      <c r="A92" s="30" t="inlineStr">
+    <row r="114" ht="18" customHeight="1">
+      <c r="A114" s="30" t="inlineStr">
         <is>
           <t>Tài khoản Google Play</t>
         </is>
       </c>
-      <c r="B92" s="15" t="n"/>
-      <c r="C92" s="31" t="inlineStr">
+      <c r="B114" s="35" t="n"/>
+      <c r="C114" s="31" t="inlineStr">
         <is>
           <t>~625.000 đ / một lần</t>
         </is>
       </c>
-      <c r="D92" s="30" t="inlineStr">
+      <c r="D114" s="30" t="inlineStr">
         <is>
           <t>Nếu phát hành Play Store</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="18" customHeight="1">
-      <c r="A93" s="27" t="inlineStr">
+    <row r="115" ht="18" customHeight="1">
+      <c r="A115" s="27" t="inlineStr">
         <is>
           <t>TỔNG ƯỚC TÍNH HÀNG THÁNG (bảo trì + VPS)</t>
         </is>
       </c>
-      <c r="B93" s="21" t="n"/>
-      <c r="C93" s="28" t="inlineStr">
+      <c r="B115" s="35" t="n"/>
+      <c r="C115" s="28" t="inlineStr">
         <is>
           <t>~5.500.000 đ / tháng</t>
         </is>
       </c>
-      <c r="D93" s="29" t="inlineStr">
+      <c r="D115" s="29" t="inlineStr">
         <is>
           <t>Chưa gồm SMS theo lượng</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="32" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="32" t="inlineStr">
         <is>
           <t>ĐẠI DIỆN KHÁCH HÀNG</t>
         </is>
       </c>
-      <c r="C96" s="32" t="inlineStr">
+      <c r="C118" s="32" t="inlineStr">
         <is>
           <t>ĐƠN VỊ PHÁT TRIỂN</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="33" t="inlineStr">
+    <row r="119">
+      <c r="A119" s="33" t="inlineStr">
         <is>
           <t>(Ký, ghi rõ họ tên)</t>
         </is>
       </c>
-      <c r="C97" s="33" t="inlineStr">
+      <c r="C119" s="33" t="inlineStr">
         <is>
           <t>(Ký, ghi rõ họ tên)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="47">
+  <mergeCells count="57">
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A92:B92"/>
+    <mergeCell ref="A106:D106"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="A75:C75"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A74:C74"/>
+    <mergeCell ref="A100:D100"/>
+    <mergeCell ref="A107:B107"/>
     <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A81:D81"/>
-    <mergeCell ref="C97:D97"/>
-    <mergeCell ref="A88:B88"/>
+    <mergeCell ref="A119:B119"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A110:B110"/>
     <mergeCell ref="A50:C50"/>
-    <mergeCell ref="A12:C12"/>
     <mergeCell ref="A57:C57"/>
-    <mergeCell ref="A87:B87"/>
+    <mergeCell ref="A95:C95"/>
+    <mergeCell ref="A102:D102"/>
     <mergeCell ref="A42:C42"/>
-    <mergeCell ref="A71:C71"/>
     <mergeCell ref="A47:C47"/>
-    <mergeCell ref="A77:D77"/>
-    <mergeCell ref="A90:B90"/>
+    <mergeCell ref="A85:C85"/>
+    <mergeCell ref="A108:B108"/>
     <mergeCell ref="A22:C22"/>
-    <mergeCell ref="A82:D82"/>
-    <mergeCell ref="A89:B89"/>
+    <mergeCell ref="A97:C97"/>
+    <mergeCell ref="A91:C91"/>
     <mergeCell ref="A53:C53"/>
+    <mergeCell ref="A118:B118"/>
+    <mergeCell ref="C118:D118"/>
     <mergeCell ref="B8:C8"/>
+    <mergeCell ref="A96:C96"/>
     <mergeCell ref="A72:C72"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A79:D79"/>
-    <mergeCell ref="A86:B86"/>
+    <mergeCell ref="A103:D103"/>
     <mergeCell ref="A44:C44"/>
-    <mergeCell ref="A78:D78"/>
-    <mergeCell ref="A85:B85"/>
+    <mergeCell ref="A93:C93"/>
+    <mergeCell ref="A113:B113"/>
+    <mergeCell ref="C119:D119"/>
+    <mergeCell ref="A92:C92"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="A59:C59"/>
-    <mergeCell ref="A73:C73"/>
-    <mergeCell ref="A84:D84"/>
-    <mergeCell ref="A91:B91"/>
-    <mergeCell ref="A97:B97"/>
-    <mergeCell ref="A80:D80"/>
-    <mergeCell ref="A96:B96"/>
+    <mergeCell ref="A99:D99"/>
+    <mergeCell ref="A109:B109"/>
+    <mergeCell ref="A82:C82"/>
     <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A94:C94"/>
+    <mergeCell ref="A112:B112"/>
+    <mergeCell ref="A105:D105"/>
     <mergeCell ref="A61:C61"/>
-    <mergeCell ref="A93:B93"/>
+    <mergeCell ref="A101:D101"/>
+    <mergeCell ref="A88:C88"/>
+    <mergeCell ref="A115:B115"/>
+    <mergeCell ref="A104:D104"/>
+    <mergeCell ref="A111:B111"/>
+    <mergeCell ref="A78:C78"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="C96:D96"/>
+    <mergeCell ref="A71:D71"/>
     <mergeCell ref="A65:C65"/>
+    <mergeCell ref="A114:B114"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>